<commit_message>
feat(infra): activate core modules and sync project board #27
</commit_message>
<xml_diff>
--- a/cells/auditor/Registro_Evaluaciones_PedagogIA.xlsx
+++ b/cells/auditor/Registro_Evaluaciones_PedagogIA.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,41 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>Calidad Técnica (4), Documentación (4), Arquitectura (4), Innovación (4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:47:47</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>test_work</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>test_work.txt</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Auditoria (rubrica_test.txt)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Insuficiente</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Criterios de Evaluación: (4), 1. Claridad en la redacción y ortografía. (4), 2. Profundidad del análisis técnico. (4), 3. Calidad de las conclusiones pedagógicas. (6), 4. Uso correcto de bibliografía. (4)</t>
         </is>
       </c>
     </row>

</xml_diff>